<commit_message>
modification code drone & new data motors
</commit_message>
<xml_diff>
--- a/motor_correction/motor power.xlsx
+++ b/motor_correction/motor power.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxime\Documents\Projet\drone\Code\Drone-code\motor_correction\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9E9D5A3B-FB87-4635-BF89-DCF31707D09B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2426FBC5-6C09-4CF1-B0C1-9BABA815A180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{72B7F52F-E4AC-4AC5-85C1-2DE790634788}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{72B7F52F-E4AC-4AC5-85C1-2DE790634788}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t>moteur A pin 9</t>
   </si>
@@ -76,12 +77,33 @@
   <si>
     <t>corr esc</t>
   </si>
+  <si>
+    <t>moteur A</t>
+  </si>
+  <si>
+    <t>moteur B</t>
+  </si>
+  <si>
+    <t>esc A</t>
+  </si>
+  <si>
+    <t>esc B</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>b</t>
+  </si>
+  <si>
+    <t>c</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +118,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -118,11 +145,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -130,6 +154,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1381,7 +1412,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="fr-FR"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2611,6 +2642,558 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="fr-FR"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="lineMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>ESCA vs ESCB</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.30683064369429069"/>
+                  <c:y val="-5.7125212289640265E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent1"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="2"/>
+            <c:dispRSqr val="1"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.3573711701878856E-2"/>
+                  <c:y val="-4.1471954014797925E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="0.0000E+00" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="fr-FR"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Feuil2!$D$2:$D$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1400</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1600</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Feuil2!$E$2:$E$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>1042</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1080</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1110</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1190</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1250</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1340</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1443</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1523</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1606</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-06E4-4BEF-AFED-FB99ED4E1FD6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:v>fonction 2nd deg</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Feuil2!$D$2:$D$10</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>1100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1150</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1200</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1300</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1400</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1500</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1600</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1700</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1800</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Feuil2!$F$2:$F$10</c:f>
+              <c:numCache>
+                <c:formatCode>0.00E+00</c:formatCode>
+                <c:ptCount val="9"/>
+                <c:pt idx="0">
+                  <c:v>1062.3767425799999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1095.03323103</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1128.51662992</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1197.9641590199999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1270.7193298799998</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1346.7821425</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1426.1525968799999</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1508.8306930200001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1594.8164309200001</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-06E4-4BEF-AFED-FB99ED4E1FD6}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="1076586015"/>
+        <c:axId val="1076586975"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="1076586015"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="1000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1076586975"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="1076586975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="1000"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="fr-FR"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1076586015"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="fr-FR"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -2731,6 +3314,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
@@ -3764,6 +4387,522 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -4384,6 +5523,47 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>571501</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>28575</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>409576</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Graphique 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{544DDB4A-B3A7-15E3-B84B-705CC1F9F62A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -4710,281 +5890,281 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B21DC9A9-6100-4C1F-A5AD-DA2A4F0544C5}">
   <dimension ref="A2:G53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
     </row>
-    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>1000</v>
       </c>
       <c r="B4">
         <v>988</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="1">
         <f>($B$4-B4)*9.81/1000</f>
         <v>0</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>1100</v>
       </c>
       <c r="B5">
         <v>988</v>
       </c>
-      <c r="C5" s="2">
+      <c r="C5" s="1">
         <f t="shared" ref="C5:C15" si="0">($B$4-B5)*9.81/1000</f>
         <v>0</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
-      <c r="E5" s="2" t="e">
-        <f>ABS((C43-C5)/C5 * 100)</f>
+      <c r="E5" s="1" t="e">
+        <f t="shared" ref="E5:E15" si="1">ABS((C43-C5)/C5 * 100)</f>
         <v>#DIV/0!</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>1150</v>
       </c>
       <c r="B6">
         <v>979</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="1">
         <f t="shared" si="0"/>
         <v>8.8290000000000007E-2</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <f>ABS((C21-C6)/C6 * 100)</f>
         <v>11.111111111111109</v>
       </c>
-      <c r="E6" s="2">
-        <f>ABS((C44-C6)/C6 * 100)</f>
+      <c r="E6" s="1">
+        <f t="shared" si="1"/>
         <v>400</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>1200</v>
       </c>
       <c r="B7">
         <v>963</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="1">
         <f t="shared" si="0"/>
         <v>0.24525</v>
       </c>
-      <c r="D7" s="2">
-        <f t="shared" ref="D7:D15" si="1">ABS((C22-C7)/C7 * 100)</f>
+      <c r="D7" s="1">
+        <f t="shared" ref="D7:D15" si="2">ABS((C22-C7)/C7 * 100)</f>
         <v>11.999999999999995</v>
       </c>
-      <c r="E7" s="2">
-        <f>ABS((C45-C7)/C7 * 100)</f>
+      <c r="E7" s="1">
+        <f t="shared" si="1"/>
         <v>144.00000000000006</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>1300</v>
       </c>
       <c r="B8">
         <v>937</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="1">
         <f t="shared" si="0"/>
         <v>0.50031000000000003</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+      <c r="E8" s="1">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="E8" s="2">
-        <f>ABS((C46-C8)/C8 * 100)</f>
         <v>74.509803921568619</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>1400</v>
       </c>
       <c r="B9">
         <v>902</v>
       </c>
-      <c r="C9" s="2">
+      <c r="C9" s="1">
         <f t="shared" si="0"/>
         <v>0.84366000000000008</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
+        <f t="shared" si="2"/>
+        <v>9.3023255813953476</v>
+      </c>
+      <c r="E9" s="1">
         <f t="shared" si="1"/>
-        <v>9.3023255813953476</v>
-      </c>
-      <c r="E9" s="2">
-        <f>ABS((C47-C9)/C9 * 100)</f>
         <v>34.883720930232556</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>1500</v>
       </c>
       <c r="B10">
         <v>892</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="1">
         <f t="shared" si="0"/>
         <v>0.94176000000000004</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
+        <f t="shared" si="2"/>
+        <v>3.1249999999999951</v>
+      </c>
+      <c r="E10" s="1">
         <f t="shared" si="1"/>
-        <v>3.1249999999999951</v>
-      </c>
-      <c r="E10" s="2">
-        <f>ABS((C48-C10)/C10 * 100)</f>
         <v>80.208333333333329</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>1600</v>
       </c>
       <c r="B11">
         <v>868</v>
       </c>
-      <c r="C11" s="2">
+      <c r="C11" s="1">
         <f t="shared" si="0"/>
         <v>1.1772</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
+        <f t="shared" si="2"/>
+        <v>8.3333333333333197</v>
+      </c>
+      <c r="E11" s="1">
         <f t="shared" si="1"/>
-        <v>8.3333333333333197</v>
-      </c>
-      <c r="E11" s="2">
-        <f>ABS((C49-C11)/C11 * 100)</f>
         <v>61.666666666666671</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>1700</v>
       </c>
       <c r="B12">
         <v>848</v>
       </c>
-      <c r="C12" s="2">
+      <c r="C12" s="1">
         <f t="shared" si="0"/>
         <v>1.3734000000000002</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
+        <f t="shared" si="2"/>
+        <v>9.2857142857142794</v>
+      </c>
+      <c r="E12" s="1">
         <f t="shared" si="1"/>
-        <v>9.2857142857142794</v>
-      </c>
-      <c r="E12" s="2">
-        <f>ABS((C50-C12)/C12 * 100)</f>
         <v>71.428571428571402</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>1800</v>
       </c>
       <c r="B13">
         <v>804</v>
       </c>
-      <c r="C13" s="2">
+      <c r="C13" s="1">
         <f t="shared" si="0"/>
         <v>1.8050400000000002</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
+        <f t="shared" si="2"/>
+        <v>2.7173913043478279</v>
+      </c>
+      <c r="E13" s="1">
         <f t="shared" si="1"/>
-        <v>2.7173913043478279</v>
-      </c>
-      <c r="E13" s="2">
-        <f>ABS((C51-C13)/C13 * 100)</f>
         <v>78.804347826086968</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>1900</v>
       </c>
       <c r="B14">
         <v>757</v>
       </c>
-      <c r="C14" s="2">
+      <c r="C14" s="1">
         <f t="shared" si="0"/>
         <v>2.2661100000000003</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
+        <f t="shared" si="2"/>
+        <v>7.3593073593073415</v>
+      </c>
+      <c r="E14" s="1">
         <f t="shared" si="1"/>
-        <v>7.3593073593073415</v>
-      </c>
-      <c r="E14" s="2">
-        <f>ABS((C52-C14)/C14 * 100)</f>
         <v>42.424242424242422</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2000</v>
       </c>
       <c r="B15">
         <v>692</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="1">
         <f t="shared" si="0"/>
         <v>2.9037600000000001</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
+        <f t="shared" si="2"/>
+        <v>5.0675675675675791</v>
+      </c>
+      <c r="E15" s="1">
         <f t="shared" si="1"/>
-        <v>5.0675675675675791</v>
-      </c>
-      <c r="E15" s="2">
-        <f>ABS((C53-C15)/C15 * 100)</f>
         <v>11.148648648648658</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>1</v>
       </c>
@@ -4995,158 +6175,158 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>1000</v>
       </c>
       <c r="B19">
         <v>988</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="1">
         <f>($B$19-B19)*9.81/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>1100</v>
       </c>
       <c r="B20">
         <v>988</v>
       </c>
-      <c r="C20" s="2">
-        <f t="shared" ref="C20:C30" si="2">($B$19-B20)*9.81/1000</f>
+      <c r="C20" s="1">
+        <f t="shared" ref="C20:C30" si="3">($B$19-B20)*9.81/1000</f>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>1150</v>
       </c>
       <c r="B21">
         <v>980</v>
       </c>
-      <c r="C21" s="2">
+      <c r="C21" s="1">
         <f>($B$19-B21)*9.81/1000</f>
         <v>7.8480000000000008E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>1200</v>
       </c>
       <c r="B22">
         <v>966</v>
       </c>
-      <c r="C22" s="2">
-        <f t="shared" si="2"/>
+      <c r="C22" s="1">
+        <f t="shared" si="3"/>
         <v>0.21582000000000001</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>1300</v>
       </c>
       <c r="B23">
         <v>937</v>
       </c>
-      <c r="C23" s="2">
-        <f t="shared" si="2"/>
+      <c r="C23" s="1">
+        <f t="shared" si="3"/>
         <v>0.50031000000000003</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>1400</v>
       </c>
       <c r="B24">
         <v>910</v>
       </c>
-      <c r="C24" s="2">
-        <f t="shared" si="2"/>
+      <c r="C24" s="1">
+        <f t="shared" si="3"/>
         <v>0.76518000000000008</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>1500</v>
       </c>
       <c r="B25">
         <v>895</v>
       </c>
-      <c r="C25" s="2">
-        <f t="shared" si="2"/>
+      <c r="C25" s="1">
+        <f t="shared" si="3"/>
         <v>0.91233000000000009</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>1600</v>
       </c>
       <c r="B26">
         <v>858</v>
       </c>
-      <c r="C26" s="2">
-        <f t="shared" si="2"/>
+      <c r="C26" s="1">
+        <f t="shared" si="3"/>
         <v>1.2752999999999999</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>1700</v>
       </c>
       <c r="B27">
         <v>835</v>
       </c>
-      <c r="C27" s="2">
-        <f t="shared" si="2"/>
+      <c r="C27" s="1">
+        <f t="shared" si="3"/>
         <v>1.5009300000000001</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>1800</v>
       </c>
       <c r="B28">
         <v>799</v>
       </c>
-      <c r="C28" s="2">
-        <f t="shared" si="2"/>
+      <c r="C28" s="1">
+        <f t="shared" si="3"/>
         <v>1.8540900000000002</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>1900</v>
       </c>
       <c r="B29">
         <v>740</v>
       </c>
-      <c r="C29" s="2">
-        <f t="shared" si="2"/>
+      <c r="C29" s="1">
+        <f t="shared" si="3"/>
         <v>2.4328799999999999</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2000</v>
       </c>
       <c r="B30">
         <v>677</v>
       </c>
-      <c r="C30" s="2">
-        <f t="shared" si="2"/>
+      <c r="C30" s="1">
+        <f t="shared" si="3"/>
         <v>3.0509100000000005</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A33" s="1" t="s">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="B33" s="1"/>
-      <c r="C33" s="1"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>1</v>
       </c>
@@ -5169,18 +6349,18 @@
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>1000</v>
       </c>
       <c r="B35">
         <v>984</v>
       </c>
-      <c r="C35" s="2">
+      <c r="C35" s="1">
         <f>($B$35-B35)*9.81/1000</f>
         <v>0</v>
       </c>
-      <c r="D35" s="2">
+      <c r="D35" s="1">
         <f>C35*E35</f>
         <v>0</v>
       </c>
@@ -5195,96 +6375,96 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>1030</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>1040</v>
       </c>
       <c r="B37">
         <v>5</v>
       </c>
-      <c r="C37" s="2">
-        <f>+B37*9.81/1000</f>
+      <c r="C37" s="1">
+        <f t="shared" ref="C37:C42" si="4">+B37*9.81/1000</f>
         <v>4.9050000000000003E-2</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>1050</v>
       </c>
       <c r="B38">
         <v>10</v>
       </c>
-      <c r="C38" s="2">
-        <f>+B38*9.81/1000</f>
+      <c r="C38" s="1">
+        <f t="shared" si="4"/>
         <v>9.8100000000000007E-2</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>1060</v>
       </c>
       <c r="B39">
         <v>15</v>
       </c>
-      <c r="C39" s="2">
-        <f>+B39*9.81/1000</f>
+      <c r="C39" s="1">
+        <f t="shared" si="4"/>
         <v>0.14715</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>1070</v>
       </c>
       <c r="B40">
         <v>20</v>
       </c>
-      <c r="C40" s="2">
-        <f>+B40*9.81/1000</f>
+      <c r="C40" s="1">
+        <f t="shared" si="4"/>
         <v>0.19620000000000001</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>1080</v>
       </c>
       <c r="B41">
         <v>25</v>
       </c>
-      <c r="C41" s="2">
-        <f>+B41*9.81/1000</f>
+      <c r="C41" s="1">
+        <f t="shared" si="4"/>
         <v>0.24525</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>1090</v>
       </c>
       <c r="B42">
         <v>30</v>
       </c>
-      <c r="C42" s="2">
-        <f>+B42*9.81/1000</f>
+      <c r="C42" s="1">
+        <f t="shared" si="4"/>
         <v>0.29430000000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>1100</v>
       </c>
       <c r="B43">
         <v>947</v>
       </c>
-      <c r="C43" s="2">
-        <f t="shared" ref="C43:C53" si="3">($B$35-B43)*9.81/1000</f>
+      <c r="C43" s="1">
+        <f t="shared" ref="C43:C51" si="5">($B$35-B43)*9.81/1000</f>
         <v>0.36297000000000001</v>
       </c>
-      <c r="D43" s="2">
-        <f>C43*E43</f>
+      <c r="D43" s="1">
+        <f t="shared" ref="D43:D53" si="6">C43*E43</f>
         <v>5.4445500000000001E-2</v>
       </c>
       <c r="E43">
@@ -5298,19 +6478,19 @@
         <v>1050</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>1150</v>
       </c>
       <c r="B44">
         <v>939</v>
       </c>
-      <c r="C44" s="2">
-        <f t="shared" si="3"/>
+      <c r="C44" s="1">
+        <f t="shared" si="5"/>
         <v>0.44145000000000006</v>
       </c>
-      <c r="D44" s="2">
-        <f>C44*E44</f>
+      <c r="D44" s="1">
+        <f t="shared" si="6"/>
         <v>0.11036250000000002</v>
       </c>
       <c r="E44">
@@ -5320,23 +6500,23 @@
         <v>0.5</v>
       </c>
       <c r="G44">
-        <f t="shared" ref="G43:G53" si="4">1000 + (A44-1000)*F44</f>
+        <f t="shared" ref="G44:G53" si="7">1000 + (A44-1000)*F44</f>
         <v>1075</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>1200</v>
       </c>
       <c r="B45">
         <v>923</v>
       </c>
-      <c r="C45" s="2">
-        <f t="shared" si="3"/>
+      <c r="C45" s="1">
+        <f t="shared" si="5"/>
         <v>0.59841000000000011</v>
       </c>
-      <c r="D45" s="2">
-        <f>C45*E45</f>
+      <c r="D45" s="1">
+        <f t="shared" si="6"/>
         <v>0.20944350000000003</v>
       </c>
       <c r="E45">
@@ -5346,23 +6526,23 @@
         <v>0.5</v>
       </c>
       <c r="G45">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1100</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>1300</v>
       </c>
       <c r="B46">
         <v>895</v>
       </c>
-      <c r="C46" s="2">
-        <f t="shared" si="3"/>
+      <c r="C46" s="1">
+        <f t="shared" si="5"/>
         <v>0.87309000000000003</v>
       </c>
-      <c r="D46" s="2">
-        <f>C46*E46</f>
+      <c r="D46" s="1">
+        <f t="shared" si="6"/>
         <v>0.43654500000000002</v>
       </c>
       <c r="E46">
@@ -5372,23 +6552,23 @@
         <v>0.5</v>
       </c>
       <c r="G46">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1150</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>1400</v>
       </c>
       <c r="B47">
         <v>868</v>
       </c>
-      <c r="C47" s="2">
-        <f t="shared" si="3"/>
+      <c r="C47" s="1">
+        <f t="shared" si="5"/>
         <v>1.1379600000000001</v>
       </c>
-      <c r="D47" s="2">
-        <f>C47*E47</f>
+      <c r="D47" s="1">
+        <f t="shared" si="6"/>
         <v>0.71691480000000007</v>
       </c>
       <c r="E47">
@@ -5398,23 +6578,23 @@
         <v>0.5</v>
       </c>
       <c r="G47">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1200</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>1500</v>
       </c>
       <c r="B48">
         <v>811</v>
       </c>
-      <c r="C48" s="2">
-        <f t="shared" si="3"/>
+      <c r="C48" s="1">
+        <f t="shared" si="5"/>
         <v>1.69713</v>
       </c>
-      <c r="D48" s="2">
-        <f>C48*E48</f>
+      <c r="D48" s="1">
+        <f t="shared" si="6"/>
         <v>1.1540484000000002</v>
       </c>
       <c r="E48">
@@ -5424,23 +6604,23 @@
         <v>0.5</v>
       </c>
       <c r="G48">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1250</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>1600</v>
       </c>
       <c r="B49">
         <v>790</v>
       </c>
-      <c r="C49" s="2">
-        <f t="shared" si="3"/>
+      <c r="C49" s="1">
+        <f t="shared" si="5"/>
         <v>1.9031400000000001</v>
       </c>
-      <c r="D49" s="2">
-        <f>C49*E49</f>
+      <c r="D49" s="1">
+        <f t="shared" si="6"/>
         <v>1.332198</v>
       </c>
       <c r="E49">
@@ -5450,23 +6630,23 @@
         <v>0.5</v>
       </c>
       <c r="G49">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1300</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>1700</v>
       </c>
       <c r="B50">
         <v>744</v>
       </c>
-      <c r="C50" s="2">
-        <f t="shared" si="3"/>
+      <c r="C50" s="1">
+        <f t="shared" si="5"/>
         <v>2.3544</v>
       </c>
-      <c r="D50" s="2">
-        <f>C50*E50</f>
+      <c r="D50" s="1">
+        <f t="shared" si="6"/>
         <v>1.64808</v>
       </c>
       <c r="E50">
@@ -5476,23 +6656,23 @@
         <v>0.5</v>
       </c>
       <c r="G50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1350</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>1800</v>
       </c>
       <c r="B51">
         <v>655</v>
       </c>
-      <c r="C51" s="2">
-        <f t="shared" si="3"/>
+      <c r="C51" s="1">
+        <f t="shared" si="5"/>
         <v>3.2274900000000004</v>
       </c>
-      <c r="D51" s="2">
-        <f>C51*E51</f>
+      <c r="D51" s="1">
+        <f t="shared" si="6"/>
         <v>2.4528924000000005</v>
       </c>
       <c r="E51">
@@ -5502,59 +6682,59 @@
         <v>0.5</v>
       </c>
       <c r="G51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1400</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>1900</v>
       </c>
       <c r="B52">
         <v>655</v>
       </c>
-      <c r="C52" s="2">
+      <c r="C52" s="1">
         <f>($B$35-B52)*9.81/1000</f>
         <v>3.2274900000000004</v>
       </c>
-      <c r="D52" s="2">
-        <f>C52*E52</f>
+      <c r="D52" s="1">
+        <f t="shared" si="6"/>
         <v>2.5174422000000005</v>
       </c>
-      <c r="E52" s="2">
+      <c r="E52" s="1">
         <v>0.78</v>
       </c>
       <c r="F52">
         <v>0.5</v>
       </c>
       <c r="G52">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1450</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2000</v>
       </c>
       <c r="B53">
         <v>655</v>
       </c>
-      <c r="C53" s="2">
+      <c r="C53" s="1">
         <f>($B$35-B53)*9.81/1000</f>
         <v>3.2274900000000004</v>
       </c>
-      <c r="D53" s="2">
-        <f>C53*E53</f>
+      <c r="D53" s="1">
+        <f t="shared" si="6"/>
         <v>2.5174422000000005</v>
       </c>
-      <c r="E53" s="2">
+      <c r="E53" s="1">
         <v>0.78</v>
       </c>
       <c r="F53">
         <v>0.5</v>
       </c>
       <c r="G53">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1500</v>
       </c>
     </row>
@@ -5568,4 +6748,230 @@
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1568BE72-E844-4B77-BFA4-7E65DF448B66}">
+  <dimension ref="A1:L10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="15" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>15</v>
+      </c>
+      <c r="K1" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="5">
+        <v>1.65382088E-4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>10</v>
+      </c>
+      <c r="B2">
+        <v>4.2</v>
+      </c>
+      <c r="D2">
+        <f>1000+A2*10</f>
+        <v>1100</v>
+      </c>
+      <c r="E2">
+        <f>1000+B2*10</f>
+        <v>1042</v>
+      </c>
+      <c r="F2" s="6">
+        <f>$L$1*D2*D2+$L$2*D2+$L$3</f>
+        <v>1062.3767425799999</v>
+      </c>
+      <c r="K2" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="5">
+        <v>0.28102007099999998</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>15</v>
+      </c>
+      <c r="B3">
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <f t="shared" ref="D3:D10" si="0">1000+A3*10</f>
+        <v>1150</v>
+      </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E10" si="1">1000+B3*10</f>
+        <v>1080</v>
+      </c>
+      <c r="F3" s="6">
+        <f t="shared" ref="F3:F10" si="2">$L$1*D3*D3+$L$2*D3+$L$3</f>
+        <v>1095.03323103</v>
+      </c>
+      <c r="K3" t="s">
+        <v>18</v>
+      </c>
+      <c r="L3" s="5">
+        <v>553.142338</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>20</v>
+      </c>
+      <c r="B4">
+        <v>11</v>
+      </c>
+      <c r="D4">
+        <f t="shared" si="0"/>
+        <v>1200</v>
+      </c>
+      <c r="E4">
+        <f t="shared" si="1"/>
+        <v>1110</v>
+      </c>
+      <c r="F4" s="6">
+        <f t="shared" si="2"/>
+        <v>1128.51662992</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>30</v>
+      </c>
+      <c r="B5">
+        <v>19</v>
+      </c>
+      <c r="D5">
+        <f t="shared" si="0"/>
+        <v>1300</v>
+      </c>
+      <c r="E5">
+        <f t="shared" si="1"/>
+        <v>1190</v>
+      </c>
+      <c r="F5" s="6">
+        <f t="shared" si="2"/>
+        <v>1197.9641590199999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>40</v>
+      </c>
+      <c r="B6">
+        <v>25</v>
+      </c>
+      <c r="D6">
+        <f t="shared" si="0"/>
+        <v>1400</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="1"/>
+        <v>1250</v>
+      </c>
+      <c r="F6" s="6">
+        <f t="shared" si="2"/>
+        <v>1270.7193298799998</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>50</v>
+      </c>
+      <c r="B7">
+        <v>34</v>
+      </c>
+      <c r="D7">
+        <f t="shared" si="0"/>
+        <v>1500</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="1"/>
+        <v>1340</v>
+      </c>
+      <c r="F7" s="6">
+        <f t="shared" si="2"/>
+        <v>1346.7821425</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>60</v>
+      </c>
+      <c r="B8">
+        <v>44.3</v>
+      </c>
+      <c r="D8">
+        <f t="shared" si="0"/>
+        <v>1600</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="1"/>
+        <v>1443</v>
+      </c>
+      <c r="F8" s="6">
+        <f t="shared" si="2"/>
+        <v>1426.1525968799999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>70</v>
+      </c>
+      <c r="B9">
+        <v>52.3</v>
+      </c>
+      <c r="D9">
+        <f t="shared" si="0"/>
+        <v>1700</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="1"/>
+        <v>1523</v>
+      </c>
+      <c r="F9" s="6">
+        <f t="shared" si="2"/>
+        <v>1508.8306930200001</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>80</v>
+      </c>
+      <c r="B10">
+        <v>60.6</v>
+      </c>
+      <c r="D10">
+        <f t="shared" si="0"/>
+        <v>1800</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="1"/>
+        <v>1606</v>
+      </c>
+      <c r="F10" s="6">
+        <f t="shared" si="2"/>
+        <v>1594.8164309200001</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>